<commit_message>
Registra prazos vencidos e guia de priorizacao por retorno financeiro
- Anota na Carneiro Machado que o processo seletivo encerrou em 30/09/2026
  e que a candidatura era so pelo formulario do site
- Aba LEIA-ME ganha secao "o que rende dinheiro mais rapido"
  (correspondencia > escritorio de volume nacional > associado remoto > RO
  local) e a lista dos prazos ja vencidos em 06/10/2026
- Orienta o posicionamento de fornecedor de comarca, nao de candidato
- Regenera o .xlsx a partir do .csv para manter os dois em sincronia

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S4PddV1zQwAFFfo7t8qVDw
</commit_message>
<xml_diff>
--- a/prospeccao_juridica/PROSPECCAO_JURIDICA_BRASIL.xlsx
+++ b/prospeccao_juridica/PROSPECCAO_JURIDICA_BRASIL.xlsx
@@ -2919,7 +2919,7 @@
       </c>
       <c r="N34" s="3" t="inlineStr">
         <is>
-          <t>DESTAQUE: vaga de ADVOGADO PREVIDENCIARISTA 100% HOME OFFICE para LIDERAR o departamento juridico. R$ 5.200 (CLT) + ajuda de custo home office + beneficios. Texto literal: "NAO HA PREFERENCIA DE LOCAL DO CANDIDATO, posto que sera home office". Sede Brasilia, atuacao nacional. E-mail nominal do responsavel pelo processo.</t>
+          <t>DESTAQUE: vaga de ADVOGADO PREVIDENCIARISTA 100% HOME OFFICE para LIDERAR o departamento juridico. R$ 5.200 (CLT) + ajuda de custo home office + beneficios. Texto literal: "NAO HA PREFERENCIA DE LOCAL DO CANDIDATO, posto que sera home office". Sede Brasilia, atuacao nacional. E-mail nominal do responsavel pelo processo. ATENCAO PRAZO: o anuncio dizia que o processo seletivo SERIA ENCERRADO EM 30/09/2026 - ja vencido. Candidatura era somente pelo formulario do site (quem ligava ou mandava WhatsApp era desclassificado). Usar este e-mail apenas para PERGUNTAR se ha vaga/cadastro ainda aberto.</t>
         </is>
       </c>
     </row>
@@ -28817,7 +28817,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -28863,7 +28863,7 @@
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>Vale enviar na segunda rodada: vaga real mas presencial, área menos aderente, ou contato institucional de escritório relevante.</t>
+          <t>Segunda rodada: vaga real mas presencial, área menos aderente, ou contato institucional de escritório relevante.</t>
         </is>
       </c>
     </row>
@@ -28875,7 +28875,7 @@
       </c>
       <c r="B7" s="15" t="inlineStr">
         <is>
-          <t>Cadastro em banco de talentos, entidade de classe, estágio ou advogado autônomo (rede/parceria, não empregador).</t>
+          <t>Banco de talentos, entidade de classe, estágio ou advogado autônomo (rede/parceria, não empregador).</t>
         </is>
       </c>
     </row>
@@ -28886,144 +28886,220 @@
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>Coluna "Confirmação" = Confirmado</t>
-        </is>
-      </c>
-      <c r="B9" s="15" t="inlineStr">
-        <is>
-          <t>O e-mail foi lido literalmente na fonte indicada na coluna Fonte (link). Pode enviar.</t>
-        </is>
-      </c>
+          <t>O QUE RENDE DINHEIRO MAIS RÁPIDO</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>Coluna "Confirmação" = Inferido</t>
+          <t>1. Correspondência</t>
         </is>
       </c>
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>ATENÇÃO — destacado em vermelho. NÃO foi lido na fonte: foi deduzido a partir de um padrão de e-mail do mesmo domínio já confirmado por um endereço real. VALIDE ANTES DE ENVIAR (teste de entrega, LinkedIn ou telefone). Não dispare em lote.</t>
+          <t>Filtre a coluna "Tipo de oportunidade" por "correspond". Pagamento por ato, começa em semanas. Seu diferencial é estar em Ji-Paraná/RO com OAB/RO ativa.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="14" t="inlineStr"/>
-      <c r="B11" s="15" t="inlineStr"/>
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>2. Escritório de volume nacional</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="inlineStr">
+        <is>
+          <t>Vá direto, sem plataforma: margem melhor. Procure na Observação por "rede", "filiais", "contencioso de massa", "bancário".</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>Regras que foram seguidas na coleta</t>
-        </is>
-      </c>
-      <c r="B12" s="15" t="inlineStr"/>
+          <t>3. Associado remoto</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>Filtre a Observação por "remoto" ou "home office". Renda recorrente.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4. Rondônia local</t>
         </is>
       </c>
       <c r="B13" s="15" t="inlineStr">
         <is>
-          <t>Nenhum e-mail foi inventado. Todo endereço "Confirmado" veio de fonte pública e verificável, com o link registrado.</t>
+          <t>Filtre Estado = RO.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="14" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B14" s="15" t="inlineStr">
-        <is>
-          <t>Somente fontes públicas e profissionais: sites oficiais, murais de vagas de subseções da OAB, portais jurídicos, anúncios de vaga em redes sociais e cadastros públicos de CNPJ.</t>
-        </is>
-      </c>
+      <c r="A14" s="14" t="inlineStr"/>
+      <c r="B14" s="15" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>Posicionamento no e-mail</t>
         </is>
       </c>
       <c r="B15" s="15" t="inlineStr">
         <is>
-          <t>Não houve acesso a bases vazadas, paywalls, contas privadas nem contorno de CAPTCHA, robots.txt ou sistema anti-bot.</t>
+          <t>Nos grupos de correspondência e parceria você NÃO é candidato, é fornecedor. Ofereça cobertura de comarca e tabela de valores — não mande currículo pedindo emprego. A taxa de resposta é muito maior.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="14" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B16" s="15" t="inlineStr">
-        <is>
-          <t>E-mails protegidos por ofuscação Cloudflare (proteção anti-robô) NÃO foram decodificados — por isso alguns escritórios aparecem na pesquisa mas não entraram na base.</t>
-        </is>
-      </c>
+      <c r="A16" s="14" t="inlineStr"/>
+      <c r="B16" s="15" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>Coluna "Confirmação" = Confirmado</t>
         </is>
       </c>
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>Nenhuma mensagem foi enviada a ninguém. Esta é apenas a fase de inteligência.</t>
+          <t>O e-mail foi lido literalmente na fonte da coluna Fonte (link). Pode enviar.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="14" t="inlineStr"/>
-      <c r="B18" s="15" t="inlineStr"/>
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>Coluna "Confirmação" = Inferido</t>
+        </is>
+      </c>
+      <c r="B18" s="15" t="inlineStr">
+        <is>
+          <t>ATENÇÃO — destacado em vermelho. NÃO foi lido na fonte: foi deduzido de um padrão de domínio já confirmado por um endereço real. VALIDE ANTES DE ENVIAR. Não inclua em disparo em lote.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="14" t="inlineStr">
-        <is>
-          <t>Antes de disparar</t>
-        </is>
-      </c>
+      <c r="A19" s="14" t="inlineStr"/>
       <c r="B19" s="15" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>Personalize</t>
-        </is>
-      </c>
-      <c r="B20" s="15" t="inlineStr">
-        <is>
-          <t>Vários anúncios exigem ASSUNTO ESPECÍFICO no e-mail (ex.: "Vaga – Advogado(a)"). Está anotado na coluna Observação. Sem o assunto correto, o currículo é descartado.</t>
-        </is>
-      </c>
+          <t>Regras seguidas na coleta</t>
+        </is>
+      </c>
+      <c r="B20" s="15" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>Cheque o prazo</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B21" s="15" t="inlineStr">
         <is>
-          <t>Algumas vagas têm data limite registrada na Observação. Confira antes de enviar.</t>
+          <t>Nenhum e-mail inventado. Todo "Confirmado" veio de fonte pública e verificável, com link registrado.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="14" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B22" s="15" t="inlineStr">
+        <is>
+          <t>Somente fontes públicas e profissionais: sites oficiais, murais de vagas de subseções da OAB, portais jurídicos, anúncios de vaga e cadastros públicos de CNPJ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="14" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B23" s="15" t="inlineStr">
+        <is>
+          <t>Sem acesso a bases vazadas, paywalls ou contas privadas; sem contornar CAPTCHA, robots.txt ou anti-bot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="inlineStr">
+        <is>
+          <t>E-mails ofuscados por Cloudflare NÃO foram decodificados — por isso alguns escritórios não entraram na base.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="14" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B25" s="15" t="inlineStr">
+        <is>
+          <t>Nenhuma mensagem foi enviada a ninguém. Esta é a fase de inteligência.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr"/>
+      <c r="B26" s="15" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
+          <t>Antes de disparar</t>
+        </is>
+      </c>
+      <c r="B27" s="15" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="14" t="inlineStr">
+        <is>
+          <t>Confira o prazo</t>
+        </is>
+      </c>
+      <c r="B28" s="15" t="inlineStr">
+        <is>
+          <t>Alguns anúncios têm data limite na Observação. Em 06/10/2026 já estavam vencidos: advogadobpa@gmail.com (Vigna), contato@cfhadvogados.com.br, andre@galdinoerebelo.com.br, contato@tcmadv.com.br e o processo da Carneiro Machado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr">
+        <is>
+          <t>Use o assunto exigido</t>
+        </is>
+      </c>
+      <c r="B29" s="15" t="inlineStr">
+        <is>
+          <t>Vários anúncios exigem assunto específico (ex.: "Vaga - Advogado(a)"). Está na Observação. Sem ele, o currículo é descartado na triagem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
           <t>Não envie em massa</t>
         </is>
       </c>
-      <c r="B22" s="15" t="inlineStr">
-        <is>
-          <t>Disparo idêntico para centenas de endereços derruba reputação do domínio e pode configurar spam. Envie em lotes pequenos e personalizados.</t>
+      <c r="B30" s="15" t="inlineStr">
+        <is>
+          <t>Disparo idêntico para centenas de endereços derruba a reputação do seu domínio. Lotes de 15 a 20 por dia, personalizados.</t>
         </is>
       </c>
     </row>

</xml_diff>